<commit_message>
Extend card sorting templates to 25 departments
Add 자동차공학과 as department #25 (the Ulsan industry boundary case
already used everywhere else in the analysis) to both card-sorting
workbooks, which were still on the 24-department scope.

- 평가: add dept row 30, extend completion formulas (/25), validation C6:C30
- 집계분석: 24x24 -> 25x25 co-occurrence matrix
- 분석용_쌍데이터: 276 -> 300 pairs (C(25,2))
- Response_QA: add Group 25 column, ranges to row 30, missing-dept check <25
- distribution: guide/PreSubmit text updated to 25 departments

Done via reproducible src/update_card_sorting_25.py.
</commit_message>
<xml_diff>
--- a/department-course-clustering/templates/card_sorting/CardSorting_distribution_individual_response.xlsx
+++ b/department-course-clustering/templates/card_sorting/CardSorting_distribution_individual_response.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>제시된 24개 학과를 "비슷한 성격의 학과끼리" 자유롭게 묶어주세요.</t>
+          <t>제시된 25개 학과를 "비슷한 성격의 학과끼리" 자유롭게 묶어주세요.</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
     <row r="3" ht="25.5" customHeight="1">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>The order and size of group numbers do not matter. Use any integers from 1 to 24.</t>
+          <t>The order and size of group numbers do not matter. Use any integers from 1 to 25.</t>
         </is>
       </c>
     </row>
@@ -1299,6 +1299,18 @@
       <c r="C29" s="36" t="n"/>
       <c r="D29" s="37" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="34" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="35" t="inlineStr">
+        <is>
+          <t>자동차공학과</t>
+        </is>
+      </c>
+      <c r="C30" s="36" t="n"/>
+      <c r="D30" s="37" t="n"/>
+    </row>
     <row r="31" ht="24.75" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
         <is>
@@ -1315,11 +1327,11 @@
         </is>
       </c>
       <c r="C32" s="17">
-        <f>COUNTA(C6:C29)/24</f>
+        <f>COUNTA(C6:C30)/25</f>
         <v/>
       </c>
       <c r="D32" s="17">
-        <f>COUNTA(D6:D29)/24</f>
+        <f>COUNTA(D6:D30)/25</f>
         <v/>
       </c>
     </row>
@@ -1331,7 +1343,7 @@
     <mergeCell ref="A1:S1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C6:C29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Check input" error="Please enter an integer from 1 to 24." promptTitle="Group number" prompt="Use the same number for departments in the same group." type="whole" operator="between">
+    <dataValidation sqref="C6:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Check input" error="Please enter an integer from 1 to 24." promptTitle="Group number" prompt="Use the same number for departments in the same group." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>24</formula2>
     </dataValidation>
@@ -1347,7 +1359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1869,6 +1881,26 @@
       <c r="D28" s="16" t="inlineStr">
         <is>
           <t>순수 화학 연구, 화학 이론</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>자동차공학과</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>공학</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>자동차 설계, 동력·구동 시스템</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1941,7 @@
     <row r="2">
       <c r="A2" s="39" t="inlineStr">
         <is>
-          <t>All 24 departments have a group number in Evaluation!C6:C29.</t>
+          <t>All 25 departments have a group number in Evaluation!C6:C30.</t>
         </is>
       </c>
       <c r="B2" s="39" t="inlineStr"/>

</xml_diff>